<commit_message>
Corrige bairro Idianópolis/Indianapolis para Indianópolis (Caruaru)
Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Hcah7c31rw93xZUdP77p41
</commit_message>
<xml_diff>
--- a/src/data/militancia/militancia-corrigido.xlsx
+++ b/src/data/militancia/militancia-corrigido.xlsx
@@ -1345,7 +1345,7 @@
         <v>Caruaru</v>
       </c>
       <c r="D56" t="str">
-        <v>Idianópolis</v>
+        <v>Indianópolis</v>
       </c>
       <c r="E56" t="str">
         <v>+55 81 9440-4019</v>
@@ -1362,7 +1362,7 @@
         <v>Caruaru</v>
       </c>
       <c r="D57" t="str">
-        <v>Indianapolis</v>
+        <v>Indianópolis</v>
       </c>
       <c r="E57" t="str">
         <v>+55 81 9653-4040</v>

</xml_diff>